<commit_message>
Fix PRTELE/CATE creation hierarchy and update test Excel
- gpartcreate: navigate to PRTWLD-TEKCATALOG before PRTELE creation
- gpartcreate: remove incorrect RecCommodity/RecSch PRTELE creation
- catecreate: navigate to CATA-TEKCATALOG before SECT creation
- Test Excel col4 (RecGpartLevel): corrected to GPART code minus last 2 chars

https://claude.ai/code/session_01PmxqqaySzGfvdiLjzyZN3E
</commit_message>
<xml_diff>
--- a/TEKCatalogGrid_TEST.xlsx
+++ b/TEKCatalogGrid_TEST.xlsx
@@ -466,7 +466,7 @@
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
@@ -557,7 +557,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>ALFBBB0BX</t>
+          <t>ALFBBB0BX00000000ZZ</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -619,7 +619,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>ALFBBB0BX</t>
+          <t>ALFBBB0BX00000000ZZ</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>ALFBBB0BX</t>
+          <t>ALFBBB0BX00000000ZZ</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>ALFBBB0BX</t>
+          <t>ALFBBB0BX00000000ZZ</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>ALCCC0BX</t>
+          <t>ALCCC0BX00000000ZZ</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Rewrite catalog hierarchy with 16-column Excel structure
PRTWLD: dynamic 5-level PRTELE (PRTWLD→P1→P2→P3→P4-COMMODITY→P5-COMwSCH→GPART)
CATA: dynamic CATA/SECT from Excel columns
- control(): new column mapping col1-16, clean variable names
- gpartcreate(): 5-level PRTELE creation, dynamic PRTWLD from col4
- catecreate(): dynamic CATA(col12) and SECT(col13)
- catescom(): renamed param RecCate→RecCateCode
- checkStatus(): updated to col1/col14/col16
- Test Excel updated to 16-column structure

https://claude.ai/code/session_01PmxqqaySzGfvdiLjzyZN3E
</commit_message>
<xml_diff>
--- a/TEKCatalogGrid_TEST.xlsx
+++ b/TEKCatalogGrid_TEST.xlsx
@@ -460,27 +460,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>GPART</t>
+          <t>GPART CODE</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -495,47 +499,67 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>GPART LEVEL</t>
+          <t>PRTWLD</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>COMMODITY</t>
+          <t>PRTELE1</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>COMMODITY DESC</t>
+          <t>PRTELE2</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>SCH</t>
+          <t>PRTELE3</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>SCH DESC</t>
+          <t>PRTELE4-COMMODITY</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>PRTELE4-COMMODITY-DESC</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>PRTELE5-COMwSCH</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>PRTELE5-COMwSCH-DESC</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>CATA</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>SECT</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>CATE</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>CATE CODE</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>CATE DESC</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>SCOM</t>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SCOM CODE</t>
         </is>
       </c>
     </row>
@@ -552,50 +576,70 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>FLANGE</t>
+          <t>FLAN</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>TEK-PRTWLD-2020</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>ANSI-API</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>A-FLAN</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>A-FLAN-WN</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>ALFBBB0BX00000000</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>ALFBBB0BX00000000ZZ</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF ASTM A105 28.58MM x 28.58MM</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>T-Pipe-Ansi-FLAN</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>T-Pipe-Ansi-FLAN-RF</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>ALFBBB0</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>ALFBBB0ZZ</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>28.58MM</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>PIPING-SECT</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>ALFBBB0</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>ALFBBB0JJ</t>
         </is>
@@ -614,50 +658,70 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>FLANGE</t>
+          <t>FLAN</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>TEK-PRTWLD-2020</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>ANSI-API</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>A-FLAN</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>A-FLAN-WN</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>ALFBBB0BX00000000</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>ALFBBB0BX00000000ZZ</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF ASTM A182 28.58MM x 28.58MM</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>T-Pipe-Ansi-FLAN</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>T-Pipe-Ansi-FLAN-RF</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>ALFBBB0</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>ALFBBB0ZZ</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>28.58MM</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>PIPING-SECT</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>ALFBBB0</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>ALFBBB0JJ</t>
         </is>
@@ -676,50 +740,70 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>FLANGE</t>
+          <t>FLAN</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
+          <t>TEK-PRTWLD-2020</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>ANSI-API</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>A-FLAN</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>A-FLAN-WN</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>ALFBBB0BX00000000</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
           <t>ALFBBB0BX00000000ZZ</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF ASTM A105 33.32MM x 33.32MM</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>T-Pipe-Ansi-FLAN</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>T-Pipe-Ansi-FLAN-RF</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>ALFBBB0</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>ALFBBB0KK</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>33.32MM</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>PIPING-SECT</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>ALFBBB0</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>ALFBBB0KK</t>
         </is>
@@ -738,50 +822,70 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>FLANGE</t>
+          <t>FLAN</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>ALFBBB0BX00000000ZZ</t>
+          <t>TEK-PRTWLD-2020</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
+          <t>ANSI-API</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>A-FLAN</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>A-FLAN-WN</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>ALFBBB0BX00000000</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>ALFBBB0BX00000000KK</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF ASTM A182 33.32MM x 33.32MM</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>T-Pipe-Ansi-FLAN</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>T-Pipe-Ansi-FLAN-RF</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
           <t>ALFBBB0</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>ALFBBB0KK</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>33.32MM</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>PIPING-SECT</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>ALFBBB0</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>BLIND FLANGE ASME B16.47 SERIES B 150# RF</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>ALFBBB0KK</t>
         </is>
@@ -800,50 +904,70 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>FLANGE</t>
+          <t>FLAN</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
+          <t>TEK-PRTWLD-2020</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>ANSI-API</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>A-FLAN</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>A-FLAN-WN</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>ALCCC0BX00000000</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>BLIND FLANGE ASME B16.47 SERIES B 300# RF</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
           <t>ALCCC0BX00000000ZZ</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>BLIND FLANGE ASME B16.47 SERIES B 300# RF ASTM A105 28.58MM x 28.58MM</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>T-Pipe-Ansi-FLAN</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>T-Pipe-Ansi-FLAN-RF</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>ALCCC0</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>BLIND FLANGE ASME B16.47 SERIES B 300# RF</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>ALCCC0ZZ</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>28.58MM</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>PIPING-SECT</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>ALCCC0</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>BLIND FLANGE ASME B16.47 SERIES B 300# RF</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>ALCCC0JJ</t>
         </is>
@@ -864,8 +988,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -876,7 +1000,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Beklenen Senaryo</t>
+          <t>Senaryo</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -891,7 +1015,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CATE=ALFBBB0 EXIST, SCOM=ALFBBB0JJ EXIST</t>
+          <t>CATE EXIST + SCOM EXIST</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -906,12 +1030,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CATE=ALFBBB0 EXIST, SCOM=ALFBBB0JJ EXIST</t>
+          <t>CATE EXIST + SCOM EXIST</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sadece GPART oluşturulur</t>
+          <t>Sadece GPART oluşturulur (farklı materyal)</t>
         </is>
       </c>
     </row>
@@ -921,7 +1045,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CATE=ALFBBB0 EXIST, SCOM=ALFBBB0KK NEW</t>
+          <t>CATE EXIST + SCOM NEW</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -936,12 +1060,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CATE=ALFBBB0 EXIST, SCOM=ALFBBB0KK NEW</t>
+          <t>CATE EXIST + SCOM EXIST</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sadece GPART oluşturulur (SCOM zaten 4. satırda yapıldı)</t>
+          <t>Sadece GPART oluşturulur (SCOM 4. satırda yapıldı)</t>
         </is>
       </c>
     </row>
@@ -951,7 +1075,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CATE=ALCCC0 NEW, SCOM=ALCCC0JJ NEW</t>
+          <t>CATE NEW + SCOM NEW</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">

</xml_diff>